<commit_message>
[fix/ASP-7990-Device-Api-Key-List-Bug] Update missing reports
</commit_message>
<xml_diff>
--- a/api/templates/export/deviceApiKeys/fr.xlsx
+++ b/api/templates/export/deviceApiKeys/fr.xlsx
@@ -1,31 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25629"/>
-  <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\export\deviceApiKeys\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2A94F9-7C64-4F9A-BC3F-CF8A3547E01F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Ключі API пристроїв" sheetId="1" r:id="rId1"/>
+    <sheet name="Ключі API пристроїв" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
-      <mx:ArchID Flags="2"/>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t xml:space="preserve">Clés API des appareils Aspect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imprimé le: &lt;date&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Table&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créé le</t>
+  </si>
+  <si>
+    <t>Clé</t>
+  </si>
+  <si>
+    <t>Partenaire</t>
+  </si>
+  <si>
+    <t>Pays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site / Appareil</t>
+  </si>
+  <si>
+    <t>Révoqué</t>
+  </si>
   <si>
     <t>&lt;createdOn&gt;</t>
   </si>
@@ -39,98 +57,59 @@
     <t>&lt;country&gt;</t>
   </si>
   <si>
-    <t>&lt;site&gt;</t>
-  </si>
-  <si>
-    <t>&lt;device&gt;</t>
+    <t>&lt;siteDevicePairsDisplay&gt;</t>
   </si>
   <si>
     <t>&lt;revoked&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Table&gt;</t>
-  </si>
-  <si>
-    <t>Ключі API пристроїв Aspect</t>
-  </si>
-  <si>
-    <t>Друкована дата: &lt;date&gt;</t>
-  </si>
-  <si>
-    <t>Створений на</t>
-  </si>
-  <si>
-    <t>Ключ</t>
-  </si>
-  <si>
-    <t>Партнер</t>
-  </si>
-  <si>
-    <t>Країна</t>
-  </si>
-  <si>
-    <t>Ділянка</t>
-  </si>
-  <si>
-    <t>Пристрій</t>
-  </si>
-  <si>
-    <t>Скасований</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
-      <sz val="12"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12.000000"/>
+      <color theme="11"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12.000000"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="16.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -144,17 +123,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="5">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="medium">
@@ -169,7 +147,7 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -184,7 +162,7 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="medium">
@@ -199,7 +177,7 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -214,136 +192,139 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="43">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="14">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf fontId="4" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="3" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="5" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="9" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="11" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="13" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="15" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="17" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="19" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9"/>
+    <cellStyle name="Followed Hyperlink" xfId="21" builtinId="9"/>
+    <cellStyle name="Hyperlink" xfId="22" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="23" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="24" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="25" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="26" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="27" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="28" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="29" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="30" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="31" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="32" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="33" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="34" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="35" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="36" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="37" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="38" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="39" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="40" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="41" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -353,7 +334,8 @@
         <i val="0"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD7D7D7"/>
           <bgColor rgb="FFD7D7D7"/>
         </patternFill>
       </fill>
@@ -364,16 +346,17 @@
         <i val="0"/>
       </font>
       <fill>
-        <patternFill patternType="none">
+        <patternFill patternType="solid">
+          <fgColor indexed="65"/>
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="0"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" table="0" pivot="0" count="2">
+      <tableStyleElement type="headerRow" size="1" dxfId="0"/>
+      <tableStyleElement type="wholeTable" size="1" dxfId="1"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -387,7 +370,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -433,13 +416,13 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -462,19 +445,18 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -497,7 +479,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -532,16 +513,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -663,9 +648,226 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
   <a:objectDefaults>
     <a:spDef>
-      <a:spPr/>
+      <a:spPr bwMode="auto"/>
       <a:bodyPr/>
       <a:lstStyle/>
       <a:style>
@@ -684,7 +886,7 @@
       </a:style>
     </a:spDef>
     <a:lnDef>
-      <a:spPr/>
+      <a:spPr bwMode="auto"/>
       <a:bodyPr/>
       <a:lstStyle/>
       <a:style>
@@ -703,107 +905,95 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="19.19921875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="31.59765625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="29.69921875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="25.8984375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="32.3984375" style="7" customWidth="1"/>
-    <col min="6" max="6" width="40.69921875" style="7" customWidth="1"/>
-    <col min="7" max="7" width="14" style="2" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" style="1" width="19.19921875"/>
+    <col customWidth="1" min="2" max="2" style="2" width="31.59765625"/>
+    <col customWidth="1" min="3" max="3" style="2" width="29.69921875"/>
+    <col customWidth="1" min="4" max="4" style="2" width="25.8984375"/>
+    <col customWidth="1" min="5" max="5" style="1" width="32.3984375"/>
+    <col customWidth="1" min="6" max="6" style="2" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="8" t="s">
-        <v>8</v>
+    <row r="1" ht="21">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>9</v>
+    <row r="2" s="1" customFormat="1">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" s="1" customFormat="1">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="4" ht="16.199999999999999">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" s="5" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>7</v>
       </c>
+      <c r="F5" s="7" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" s="3" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+    <row r="6" s="2" customFormat="1">
+      <c r="A6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C6" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E6" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>16</v>
-      </c>
     </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="12"/>
+    <row r="8">
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="13"/>
     </row>
   </sheetData>
+  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="4294967292" verticalDpi="4294967292" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>